<commit_message>
Replace bad row data in .review files with the word 'review'
</commit_message>
<xml_diff>
--- a/output/campaign_Vive_Living.review.xlsx
+++ b/output/campaign_Vive_Living.review.xlsx
@@ -413,67 +413,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Apellidos</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Números</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Nombre del proyecto</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Contacto ID</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Negocio ID</t>
+          <t>review</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Laura</t>
+          <t>review</t>
         </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Martinez</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>573043460864</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>VIVE LIVING</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>165270501</v>
-      </c>
-      <c r="F2" t="n">
-        <v>60539594514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>